<commit_message>
fix: preserve pivot table filters during save (ClosedXML/ClosedXML#2219)
The pivot cache writer always hardcoded refreshOnLoad=true, causing Excel
to rebuild the pivot table on open and discard all applied filters (hidden
items). Now the writer uses the actual RefreshDataOnOpen property value,
which is loaded from the file and defaults to true only for new caches.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Other/PivotTable/Sources/PivotTable-AllSources-output.xlsx
+++ b/XLibur.Tests/Resource/Other/PivotTable/Sources/PivotTable-AllSources-output.xlsx
@@ -308,7 +308,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="1" refreshedBy="Jan Havlíček" refreshedDate="45640.183021412035" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{5A3793E0-F24E-4218-978B-ED3C8CBB3606}" mc:Ignorable="xr">
+<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="0" refreshedBy="Jan Havlíček" refreshedDate="45640.183021412035" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{5A3793E0-F24E-4218-978B-ED3C8CBB3606}" mc:Ignorable="xr">
   <x:cacheSource type="worksheet">
     <x:worksheetSource ref="D3:E4" sheet="Area Source"/>
   </x:cacheSource>
@@ -329,7 +329,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="1" refreshedBy="Jan Havlíček" refreshedDate="45640.18319664352" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{99F43060-B546-41D9-8AD6-43E3D15EE121}" mc:Ignorable="xr">
+<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="0" refreshedBy="Jan Havlíček" refreshedDate="45640.18319664352" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{99F43060-B546-41D9-8AD6-43E3D15EE121}" mc:Ignorable="xr">
   <x:cacheSource type="worksheet">
     <x:worksheetSource name="Table1"/>
   </x:cacheSource>
@@ -350,7 +350,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="1" refreshedBy="Jan Havlíček" refreshedDate="45640.183633217595" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{1DDB9D54-7888-42ED-9CF2-85B827247CCD}" mc:Ignorable="xr">
+<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="0" refreshedBy="Jan Havlíček" refreshedDate="45640.183633217595" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{1DDB9D54-7888-42ED-9CF2-85B827247CCD}" mc:Ignorable="xr">
   <x:cacheSource type="worksheet">
     <x:worksheetSource name="AreaName"/>
   </x:cacheSource>
@@ -371,7 +371,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="1" refreshedBy="Jan Havlíček" refreshedDate="45640.19502673611" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="2" xr:uid="{D6103DA1-26CC-456C-A3F0-D133DC8655B9}" mc:Ignorable="xr">
+<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="0" refreshedBy="Jan Havlíček" refreshedDate="45640.19502673611" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="2" xr:uid="{D6103DA1-26CC-456C-A3F0-D133DC8655B9}" mc:Ignorable="xr">
   <x:cacheSource type="worksheet">
     <x:worksheetSource ref="A1:B3" sheet="Sheet1" r:id="rId2"/>
   </x:cacheSource>
@@ -392,7 +392,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="1" refreshedBy="Jan Havlíček" refreshedDate="45640.820318865743" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="2" xr:uid="{08AFD5F3-EF3C-4277-9EC0-BC5F6E36BD65}" mc:Ignorable="xr">
+<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="0" refreshedBy="Jan Havlíček" refreshedDate="45640.820318865743" backgroundQuery="1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="2" xr:uid="{08AFD5F3-EF3C-4277-9EC0-BC5F6E36BD65}" mc:Ignorable="xr">
   <x:cacheSource type="external" connectionId="1"/>
   <x:cacheFields count="2">
     <x:cacheField name="Name">
@@ -417,7 +417,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" saveData="0" refreshOnLoad="1" refreshedBy="Jan Havlíček" refreshedDate="45640.931218171296" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="2" xr:uid="{9BD42A5F-5A0C-417E-AEDF-DBA25499EC16}" mc:Ignorable="xr">
+<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" saveData="0" refreshOnLoad="0" refreshedBy="Jan Havlíček" refreshedDate="45640.931218171296" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="2" xr:uid="{9BD42A5F-5A0C-417E-AEDF-DBA25499EC16}" mc:Ignorable="xr">
   <x:cacheSource type="scenario"/>
   <x:cacheFields count="3">
     <x:cacheField name="$B$2:$B$3">
@@ -447,7 +447,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="1" refreshedBy="Jan Havlíček" refreshedDate="45641.123992361114" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{C4D000D4-C547-41E9-B0B9-2D56DCDF4F13}" mc:Ignorable="xr">
+<x:pivotCacheDefinition xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r:id="rId1" saveData="1" refreshOnLoad="0" refreshedBy="Jan Havlíček" refreshedDate="45641.123992361114" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{C4D000D4-C547-41E9-B0B9-2D56DCDF4F13}" mc:Ignorable="xr">
   <x:cacheSource type="consolidation">
     <x:consolidation autoPage="0">
       <x:pages>

</xml_diff>

<commit_message>
fix(io): read a pivot table's show-last-column emphasis from its own attribute
The reader set ShowLastColumn from the column-stripes attribute instead of its own
showLastColumn attribute, so the two settings could not vary independently: a file
with stripes on and last-column emphasis off re-saved with the emphasis switched on.

Regression test: ShowLastColumn_reads_from_its_own_attribute_not_column_stripes.
Also updates the golden pivot fixtures whose source files set showLastColumn
independently of showColStripes and therefore round-tripped incorrectly before this fix.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Other/PivotTable/Sources/PivotTable-AllSources-output.xlsx
+++ b/XLibur.Tests/Resource/Other/PivotTable/Sources/PivotTable-AllSources-output.xlsx
@@ -645,7 +645,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1"/>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition enableEdit="0" hideValuesRow="1"/>
@@ -661,7 +661,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1"/>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition enableEdit="0" hideValuesRow="1"/>
@@ -677,7 +677,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1"/>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition enableEdit="0" hideValuesRow="1"/>
@@ -693,7 +693,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1"/>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition enableEdit="0" hideValuesRow="1"/>
@@ -709,7 +709,7 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1"/>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition enableEdit="0" hideValuesRow="1"/>
@@ -756,7 +756,7 @@
   <dataFields count="1">
     <dataField name="$B$5" fld="2" baseField="0" baseItem="0"/>
   </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1"/>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition enableEdit="0" hideValuesRow="1"/>
@@ -834,7 +834,7 @@
   <dataFields count="1">
     <dataField name="Sum of Value" fld="2" baseField="0" baseItem="0"/>
   </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1"/>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
       <x14:pivotTableDefinition enableEdit="0" hideValuesRow="1"/>

</xml_diff>